<commit_message>
Updated CAN model - 2025-09-11 17:44
</commit_message>
<xml_diff>
--- a/VerveStacks_CAN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_CAN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CAN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{70B28A6D-745B-49BA-9CCB-5B2DD6B0DD7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CB5D7290-063D-4D21-9107-A87996296092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -970,18 +970,18 @@
     <t>onshore wind resource -- CF class won-CAN_52 -- cost class 2</t>
   </si>
   <si>
+    <t>e_won-CAN_51_c2</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-CAN_51 -- cost class 2</t>
+  </si>
+  <si>
     <t>e_won-CAN_51_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-CAN_51 -- cost class 1</t>
   </si>
   <si>
-    <t>e_won-CAN_51_c2</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-CAN_51 -- cost class 2</t>
-  </si>
-  <si>
     <t>e_won-CAN_51_c3</t>
   </si>
   <si>
@@ -994,16 +994,16 @@
     <t>onshore wind resource -- CF class won-CAN_50 -- cost class 4</t>
   </si>
   <si>
+    <t>e_won-CAN_50_c1</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-CAN_50 -- cost class 1</t>
+  </si>
+  <si>
     <t>e_won-CAN_50_c3</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-CAN_50 -- cost class 3</t>
-  </si>
-  <si>
-    <t>e_won-CAN_50_c1</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-CAN_50 -- cost class 1</t>
   </si>
   <si>
     <t>e_won-CAN_50_c2</t>
@@ -8370,7 +8370,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FC7DC17-BDE3-4B82-A44A-BABD7FBD88F8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51380E68-6098-41E5-A0E1-2D8B0E96D60D}">
   <dimension ref="B9:N45"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9756,7 +9756,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26625211-86AF-4658-B467-1610080E5FDC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6558944F-D20D-4D99-BB98-ED4823522E44}">
   <dimension ref="B9:AB238"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10617,13 +10617,13 @@
         <v>644</v>
       </c>
       <c r="L21">
-        <v>0.15461990569215225</v>
+        <v>0.67140036783358703</v>
       </c>
       <c r="M21">
         <v>0.51</v>
       </c>
       <c r="N21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P21" t="s">
         <v>182</v>
@@ -10691,13 +10691,13 @@
         <v>644</v>
       </c>
       <c r="L22">
-        <v>0.67140036783358703</v>
+        <v>0.15461990569215225</v>
       </c>
       <c r="M22">
         <v>0.51</v>
       </c>
       <c r="N22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P22" t="s">
         <v>182</v>
@@ -10913,13 +10913,13 @@
         <v>644</v>
       </c>
       <c r="L25">
-        <v>0.43772455768920937</v>
+        <v>7.5000000000000002E-4</v>
       </c>
       <c r="M25">
         <v>0.496</v>
       </c>
       <c r="N25">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P25" t="s">
         <v>182</v>
@@ -10987,13 +10987,13 @@
         <v>644</v>
       </c>
       <c r="L26">
-        <v>7.5000000000000002E-4</v>
+        <v>0.43772455768920937</v>
       </c>
       <c r="M26">
         <v>0.496</v>
       </c>
       <c r="N26">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P26" t="s">
         <v>182</v>
@@ -25430,7 +25430,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B060D03-267C-4A34-AD82-B60C988A4968}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DA24D5D-D542-4283-9BE2-23693F39B86C}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CAN model - 2025-09-11 17:51
</commit_message>
<xml_diff>
--- a/VerveStacks_CAN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_CAN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CAN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CB5D7290-063D-4D21-9107-A87996296092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{13499F43-4D22-454B-B115-97C761A890C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -970,18 +970,18 @@
     <t>onshore wind resource -- CF class won-CAN_52 -- cost class 2</t>
   </si>
   <si>
+    <t>e_won-CAN_51_c1</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-CAN_51 -- cost class 1</t>
+  </si>
+  <si>
     <t>e_won-CAN_51_c2</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-CAN_51 -- cost class 2</t>
   </si>
   <si>
-    <t>e_won-CAN_51_c1</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-CAN_51 -- cost class 1</t>
-  </si>
-  <si>
     <t>e_won-CAN_51_c3</t>
   </si>
   <si>
@@ -994,16 +994,16 @@
     <t>onshore wind resource -- CF class won-CAN_50 -- cost class 4</t>
   </si>
   <si>
+    <t>e_won-CAN_50_c3</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-CAN_50 -- cost class 3</t>
+  </si>
+  <si>
     <t>e_won-CAN_50_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-CAN_50 -- cost class 1</t>
-  </si>
-  <si>
-    <t>e_won-CAN_50_c3</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-CAN_50 -- cost class 3</t>
   </si>
   <si>
     <t>e_won-CAN_50_c2</t>
@@ -8370,7 +8370,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51380E68-6098-41E5-A0E1-2D8B0E96D60D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64830FC4-A3A4-4738-82D6-14AAF699BBD2}">
   <dimension ref="B9:N45"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9756,7 +9756,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6558944F-D20D-4D99-BB98-ED4823522E44}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BA297DA-3FF4-4A6A-B662-A6FA1B03CD92}">
   <dimension ref="B9:AB238"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10617,13 +10617,13 @@
         <v>644</v>
       </c>
       <c r="L21">
-        <v>0.67140036783358703</v>
+        <v>0.15461990569215225</v>
       </c>
       <c r="M21">
         <v>0.51</v>
       </c>
       <c r="N21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P21" t="s">
         <v>182</v>
@@ -10691,13 +10691,13 @@
         <v>644</v>
       </c>
       <c r="L22">
-        <v>0.15461990569215225</v>
+        <v>0.67140036783358703</v>
       </c>
       <c r="M22">
         <v>0.51</v>
       </c>
       <c r="N22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P22" t="s">
         <v>182</v>
@@ -10913,13 +10913,13 @@
         <v>644</v>
       </c>
       <c r="L25">
-        <v>7.5000000000000002E-4</v>
+        <v>0.43772455768920937</v>
       </c>
       <c r="M25">
         <v>0.496</v>
       </c>
       <c r="N25">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P25" t="s">
         <v>182</v>
@@ -10987,13 +10987,13 @@
         <v>644</v>
       </c>
       <c r="L26">
-        <v>0.43772455768920937</v>
+        <v>7.5000000000000002E-4</v>
       </c>
       <c r="M26">
         <v>0.496</v>
       </c>
       <c r="N26">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P26" t="s">
         <v>182</v>
@@ -25430,7 +25430,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DA24D5D-D542-4283-9BE2-23693F39B86C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D60A164C-B1A3-4805-8B14-6BAC877EAA9F}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CAN model - 2025-09-11 17:58
</commit_message>
<xml_diff>
--- a/VerveStacks_CAN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_CAN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CAN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{13499F43-4D22-454B-B115-97C761A890C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E722E0EC-7E9A-4811-BEEA-173C43821D8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1000,16 +1000,16 @@
     <t>onshore wind resource -- CF class won-CAN_50 -- cost class 3</t>
   </si>
   <si>
+    <t>e_won-CAN_50_c2</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-CAN_50 -- cost class 2</t>
+  </si>
+  <si>
     <t>e_won-CAN_50_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-CAN_50 -- cost class 1</t>
-  </si>
-  <si>
-    <t>e_won-CAN_50_c2</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-CAN_50 -- cost class 2</t>
   </si>
   <si>
     <t>e_won-CAN_49_c4</t>
@@ -8370,7 +8370,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64830FC4-A3A4-4738-82D6-14AAF699BBD2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D8ABE39-F8FB-4578-A0A7-9C0EAAC166A2}">
   <dimension ref="B9:N45"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9756,7 +9756,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BA297DA-3FF4-4A6A-B662-A6FA1B03CD92}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2265226A-AA2B-455B-AB40-323FFDE87C6A}">
   <dimension ref="B9:AB238"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10987,13 +10987,13 @@
         <v>644</v>
       </c>
       <c r="L26">
-        <v>7.5000000000000002E-4</v>
+        <v>0.8973618392340873</v>
       </c>
       <c r="M26">
         <v>0.496</v>
       </c>
       <c r="N26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P26" t="s">
         <v>182</v>
@@ -11061,13 +11061,13 @@
         <v>644</v>
       </c>
       <c r="L27">
-        <v>0.8973618392340873</v>
+        <v>7.5000000000000002E-4</v>
       </c>
       <c r="M27">
         <v>0.496</v>
       </c>
       <c r="N27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P27" t="s">
         <v>182</v>
@@ -25430,7 +25430,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D60A164C-B1A3-4805-8B14-6BAC877EAA9F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF05A3E5-6359-48CF-9B5E-3AF3F9A6428A}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CAN model - 2025-09-11 18:26
</commit_message>
<xml_diff>
--- a/VerveStacks_CAN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_CAN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CAN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E722E0EC-7E9A-4811-BEEA-173C43821D8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ECC34CE4-4680-4F81-90F7-6B2E86B085DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -970,18 +970,18 @@
     <t>onshore wind resource -- CF class won-CAN_52 -- cost class 2</t>
   </si>
   <si>
+    <t>e_won-CAN_51_c2</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-CAN_51 -- cost class 2</t>
+  </si>
+  <si>
     <t>e_won-CAN_51_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-CAN_51 -- cost class 1</t>
   </si>
   <si>
-    <t>e_won-CAN_51_c2</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-CAN_51 -- cost class 2</t>
-  </si>
-  <si>
     <t>e_won-CAN_51_c3</t>
   </si>
   <si>
@@ -1000,16 +1000,16 @@
     <t>onshore wind resource -- CF class won-CAN_50 -- cost class 3</t>
   </si>
   <si>
+    <t>e_won-CAN_50_c1</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-CAN_50 -- cost class 1</t>
+  </si>
+  <si>
     <t>e_won-CAN_50_c2</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-CAN_50 -- cost class 2</t>
-  </si>
-  <si>
-    <t>e_won-CAN_50_c1</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-CAN_50 -- cost class 1</t>
   </si>
   <si>
     <t>e_won-CAN_49_c4</t>
@@ -8370,7 +8370,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D8ABE39-F8FB-4578-A0A7-9C0EAAC166A2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07F1789D-877E-44A6-BE27-998F4EC72668}">
   <dimension ref="B9:N45"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9756,7 +9756,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2265226A-AA2B-455B-AB40-323FFDE87C6A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F924C147-CE01-440A-8720-FDC7528486E2}">
   <dimension ref="B9:AB238"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10617,13 +10617,13 @@
         <v>644</v>
       </c>
       <c r="L21">
-        <v>0.15461990569215225</v>
+        <v>0.67140036783358703</v>
       </c>
       <c r="M21">
         <v>0.51</v>
       </c>
       <c r="N21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P21" t="s">
         <v>182</v>
@@ -10691,13 +10691,13 @@
         <v>644</v>
       </c>
       <c r="L22">
-        <v>0.67140036783358703</v>
+        <v>0.15461990569215225</v>
       </c>
       <c r="M22">
         <v>0.51</v>
       </c>
       <c r="N22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P22" t="s">
         <v>182</v>
@@ -10987,13 +10987,13 @@
         <v>644</v>
       </c>
       <c r="L26">
-        <v>0.8973618392340873</v>
+        <v>7.5000000000000002E-4</v>
       </c>
       <c r="M26">
         <v>0.496</v>
       </c>
       <c r="N26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P26" t="s">
         <v>182</v>
@@ -11061,13 +11061,13 @@
         <v>644</v>
       </c>
       <c r="L27">
-        <v>7.5000000000000002E-4</v>
+        <v>0.8973618392340873</v>
       </c>
       <c r="M27">
         <v>0.496</v>
       </c>
       <c r="N27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P27" t="s">
         <v>182</v>
@@ -25430,7 +25430,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF05A3E5-6359-48CF-9B5E-3AF3F9A6428A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C76721B-11EE-4B85-A29C-231044DC0A6A}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CAN model - 2025-09-11 18:38
</commit_message>
<xml_diff>
--- a/VerveStacks_CAN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_CAN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CAN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ECC34CE4-4680-4F81-90F7-6B2E86B085DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BD523275-80D8-45FC-BF2C-DF151201B77B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1000,16 +1000,16 @@
     <t>onshore wind resource -- CF class won-CAN_50 -- cost class 3</t>
   </si>
   <si>
+    <t>e_won-CAN_50_c2</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-CAN_50 -- cost class 2</t>
+  </si>
+  <si>
     <t>e_won-CAN_50_c1</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-CAN_50 -- cost class 1</t>
-  </si>
-  <si>
-    <t>e_won-CAN_50_c2</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-CAN_50 -- cost class 2</t>
   </si>
   <si>
     <t>e_won-CAN_49_c4</t>
@@ -8370,7 +8370,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07F1789D-877E-44A6-BE27-998F4EC72668}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCD1E7EF-34C9-4767-B344-6F905ACABE4D}">
   <dimension ref="B9:N45"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9756,7 +9756,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F924C147-CE01-440A-8720-FDC7528486E2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABA64324-7B66-4205-BF6D-5F425083766B}">
   <dimension ref="B9:AB238"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10987,13 +10987,13 @@
         <v>644</v>
       </c>
       <c r="L26">
-        <v>7.5000000000000002E-4</v>
+        <v>0.8973618392340873</v>
       </c>
       <c r="M26">
         <v>0.496</v>
       </c>
       <c r="N26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P26" t="s">
         <v>182</v>
@@ -11061,13 +11061,13 @@
         <v>644</v>
       </c>
       <c r="L27">
-        <v>0.8973618392340873</v>
+        <v>7.5000000000000002E-4</v>
       </c>
       <c r="M27">
         <v>0.496</v>
       </c>
       <c r="N27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P27" t="s">
         <v>182</v>
@@ -25430,7 +25430,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C76721B-11EE-4B85-A29C-231044DC0A6A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5BC63D2-54CA-4A37-A8C6-E8A27FA33C05}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CAN model - 2025-09-11 22:28
</commit_message>
<xml_diff>
--- a/VerveStacks_CAN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_CAN/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CAN\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BD523275-80D8-45FC-BF2C-DF151201B77B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5123AF96-B3D2-4375-85ED-AF6028D47F5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -970,16 +970,16 @@
     <t>onshore wind resource -- CF class won-CAN_52 -- cost class 2</t>
   </si>
   <si>
+    <t>e_won-CAN_51_c1</t>
+  </si>
+  <si>
+    <t>onshore wind resource -- CF class won-CAN_51 -- cost class 1</t>
+  </si>
+  <si>
     <t>e_won-CAN_51_c2</t>
   </si>
   <si>
     <t>onshore wind resource -- CF class won-CAN_51 -- cost class 2</t>
-  </si>
-  <si>
-    <t>e_won-CAN_51_c1</t>
-  </si>
-  <si>
-    <t>onshore wind resource -- CF class won-CAN_51 -- cost class 1</t>
   </si>
   <si>
     <t>e_won-CAN_51_c3</t>
@@ -8370,7 +8370,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCD1E7EF-34C9-4767-B344-6F905ACABE4D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDA5D5F4-953D-4FE6-9CFF-13298D30D4A2}">
   <dimension ref="B9:N45"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9756,7 +9756,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABA64324-7B66-4205-BF6D-5F425083766B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB79E42B-E23F-4FED-BE89-A0C5D81781DC}">
   <dimension ref="B9:AB238"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10617,13 +10617,13 @@
         <v>644</v>
       </c>
       <c r="L21">
-        <v>0.67140036783358703</v>
+        <v>0.15461990569215225</v>
       </c>
       <c r="M21">
         <v>0.51</v>
       </c>
       <c r="N21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P21" t="s">
         <v>182</v>
@@ -10691,13 +10691,13 @@
         <v>644</v>
       </c>
       <c r="L22">
-        <v>0.15461990569215225</v>
+        <v>0.67140036783358703</v>
       </c>
       <c r="M22">
         <v>0.51</v>
       </c>
       <c r="N22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P22" t="s">
         <v>182</v>
@@ -25430,7 +25430,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5BC63D2-54CA-4A37-A8C6-E8A27FA33C05}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B9AC993-C7A5-4F90-BC0E-F901F3E4D370}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>